<commit_message>
Refatoração de scripts de automação para melhor tratamento de erros e registro de logs
- Adição de um novo módulo, `etapa.py`, para gerenciar etapas da automação e o tratamento de erros.
- Aprimoramento da função `clicar_imagem` para salvar capturas de tela em caso de falha.
- Atualização de `consumo.py` para utilizar as novas funções do módulo `etapa`, visando melhor estrutura e legibilidade.
- Modificação de `mover_e_renomear_arquivo_baixado.py` para permitir a especificação de um arquivo para renomeação.
- Melhoria das mensagens de erro e do registro de logs em todo o processo de automação.
</commit_message>
<xml_diff>
--- a/log/log_automacao.xlsx
+++ b/log/log_automacao.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$205</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7888,8 +7888,808 @@
         <v>136.7</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:18:39</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:20:05</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010009_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="n">
+        <v>85.3</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:20:05</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:21:27</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010010_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="n">
+        <v>82.59999999999999</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:21:28</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:22:51</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010034_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="n">
+        <v>83.8</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:22:52</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:23:44</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G189" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção selecionada para exportar planilha</t>
+        </is>
+      </c>
+      <c r="H189" s="4" t="n">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:29:55</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:31:28</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010040_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="n">
+        <v>93.09999999999999</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:31:28</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:32:51</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010044_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="n">
+        <v>82.90000000000001</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:32:51</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:34:15</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010057_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n">
+        <v>83.8</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:34:15</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:35:39</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010011_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="n">
+        <v>83.90000000000001</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:35:39</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:37:11</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010024_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="n">
+        <v>91.8</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:37:11</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:38:04</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G195" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção selecionada para exportar planilha</t>
+        </is>
+      </c>
+      <c r="H195" s="4" t="n">
+        <v>53.2</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:47:33</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:48:57</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010027_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:48:57</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:50:19</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010028_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="n">
+        <v>81.90000000000001</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:50:20</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:51:43</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010035_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="n">
+        <v>83.5</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:51:43</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:53:05</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010037_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="n">
+        <v>81.8</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:53:05</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:54:29</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010038_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="n">
+        <v>83.8</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:54:29</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 12:55:42</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F201" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G201" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção diretório</t>
+        </is>
+      </c>
+      <c r="H201" s="4" t="n">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:02:42</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:04:03</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010039_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="n">
+        <v>80.7</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:04:03</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:05:13</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F203" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G203" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção diretório</t>
+        </is>
+      </c>
+      <c r="H203" s="4" t="n">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:09:55</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:11:19</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010048_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="n">
+        <v>83.8</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:11:19</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:12:40</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010041_31-07-2026.csv</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H185"/>
+  <autoFilter ref="A1:H205"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona novas funções para gerenciar filiais pendentes e executar relatórios de consumo e centro de custo
</commit_message>
<xml_diff>
--- a/log/log_automacao.xlsx
+++ b/log/log_automacao.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H205"/>
+  <dimension ref="A1:H237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8688,8 +8688,1288 @@
         <v>81.59999999999999</v>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:42:10</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:44:34</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="n">
+        <v>144.9</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:44:34</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:47:00</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="n">
+        <v>145.7</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:47:00</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:49:29</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="n">
+        <v>148.6</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:49:29</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:52:38</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="n">
+        <v>189.6</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:52:38</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:55:04</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="n">
+        <v>145.5</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:55:04</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:57:27</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="n">
+        <v>143.3</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:57:27</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:59:51</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 10:59:51</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:02:15</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:02:15</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:04:39</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:04:39</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:07:09</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="n">
+        <v>150.2</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:07:09</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:09:32</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="n">
+        <v>143.1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:09:32</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:11:56</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="n">
+        <v>143.4</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:11:56</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:14:20</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:14:20</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:16:43</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="n">
+        <v>142.8</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:16:43</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:20:37</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G220" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar o tipo ponto e virgula | Não foi possível voltar para a tela inicial do relatório</t>
+        </is>
+      </c>
+      <c r="H220" s="4" t="n">
+        <v>233.9</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:20:37</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:20:37</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E221" s="4" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F221" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G221" s="4" t="inlineStr">
+        <is>
+          <t>Não processada: Não foi possível voltar para a tela inicial do relatório</t>
+        </is>
+      </c>
+      <c r="H221" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E222" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F222" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G222" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H222" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E223" s="4" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F223" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G223" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H223" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E224" s="4" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F224" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G224" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H224" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E225" s="4" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F225" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G225" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H225" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F226" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G226" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H226" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E227" s="4" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F227" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G227" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H227" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E228" s="4" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F228" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H228" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F229" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G229" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H229" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F230" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H230" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E231" s="4" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F231" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G231" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H231" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F232" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G232" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H232" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F233" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G233" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H233" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E234" s="4" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F234" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G234" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H234" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F235" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G235" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H235" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E236" s="4" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F236" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G236" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H236" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:21:45</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D237" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E237" s="4" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F237" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G237" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar o menu Relatórios</t>
+        </is>
+      </c>
+      <c r="H237" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H205"/>
+  <autoFilter ref="A1:H237"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>